<commit_message>
chore(data-release): publish site data 2026-08-14 08:57:51 UTC
</commit_message>
<xml_diff>
--- a/countries/ch/2026-2029.xlsx
+++ b/countries/ch/2026-2029.xlsx
@@ -9442,13 +9442,13 @@
         </is>
       </c>
       <c r="N61" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O61" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="R61" t="n">
-        <v>0.954728336492448</v>
+        <v>0.9658298287772439</v>
       </c>
       <c r="S61" t="inlineStr">
         <is>
@@ -14354,13 +14354,13 @@
         </is>
       </c>
       <c r="N94" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="O94" t="n">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="R94" t="n">
-        <v>2.897489486331732</v>
+        <v>2.908590978616528</v>
       </c>
       <c r="S94" t="inlineStr">
         <is>
@@ -14789,13 +14789,13 @@
         </is>
       </c>
       <c r="N97" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="O97" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="R97" t="n">
-        <v>1.187859674473162</v>
+        <v>1.210062659042754</v>
       </c>
       <c r="S97" t="inlineStr">
         <is>
@@ -19973,13 +19973,13 @@
         </is>
       </c>
       <c r="N132" t="n">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="O132" t="n">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="R132" t="n">
-        <v>4.351784975639996</v>
+        <v>4.362886467924791</v>
       </c>
       <c r="S132" t="inlineStr">
         <is>
@@ -20408,13 +20408,13 @@
         </is>
       </c>
       <c r="N135" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="O135" t="n">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="R135" t="n">
-        <v>1.198961166757958</v>
+        <v>1.232265643612346</v>
       </c>
       <c r="S135" t="inlineStr">
         <is>
@@ -24571,13 +24571,13 @@
         </is>
       </c>
       <c r="N163" t="n">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="O163" t="n">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="R163" t="n">
-        <v>9.680501272342031</v>
+        <v>9.702704256911622</v>
       </c>
       <c r="S163" t="inlineStr">
         <is>
@@ -25006,13 +25006,13 @@
         </is>
       </c>
       <c r="N166" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="O166" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="R166" t="n">
-        <v>1.46539698159306</v>
+        <v>1.476498473877856</v>
       </c>
       <c r="S166" t="inlineStr">
         <is>
@@ -26746,13 +26746,13 @@
         </is>
       </c>
       <c r="N178" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O178" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R178" t="n">
-        <v>0.05550746142397953</v>
+        <v>0.07771044599357135</v>
       </c>
       <c r="S178" t="inlineStr">
         <is>
@@ -27471,13 +27471,13 @@
         </is>
       </c>
       <c r="N183" t="n">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="O183" t="n">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="R183" t="n">
-        <v>12.15613405185152</v>
+        <v>12.16723554413631</v>
       </c>
       <c r="S183" t="inlineStr">
         <is>
@@ -27761,13 +27761,13 @@
         </is>
       </c>
       <c r="N185" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="O185" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R185" t="n">
-        <v>0.2442328302655099</v>
+        <v>0.2553343225503059</v>
       </c>
       <c r="S185" t="inlineStr">
         <is>
@@ -28196,13 +28196,13 @@
         </is>
       </c>
       <c r="N188" t="n">
-        <v>2137</v>
+        <v>2143</v>
       </c>
       <c r="O188" t="n">
-        <v>2137</v>
+        <v>2143</v>
       </c>
       <c r="R188" t="n">
-        <v>23.72388901260885</v>
+        <v>23.79049796631763</v>
       </c>
       <c r="S188" t="inlineStr">
         <is>
@@ -28486,13 +28486,13 @@
         </is>
       </c>
       <c r="N190" t="n">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="O190" t="n">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="R190" t="n">
-        <v>1.831746226991325</v>
+        <v>1.887253688415304</v>
       </c>
       <c r="S190" t="inlineStr">
         <is>
@@ -28631,13 +28631,13 @@
         </is>
       </c>
       <c r="N191" t="n">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="O191" t="n">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="R191" t="n">
-        <v>1.70962981185857</v>
+        <v>1.820644734706529</v>
       </c>
       <c r="S191" t="inlineStr">
         <is>
@@ -28994,6 +28994,1166 @@
         </is>
       </c>
       <c r="BC193" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>D004</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>COVID-19</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>新型冠状病毒感染</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N194" t="n">
+        <v>57</v>
+      </c>
+      <c r="O194" t="n">
+        <v>57</v>
+      </c>
+      <c r="R194" t="n">
+        <v>0.6327850602333667</v>
+      </c>
+      <c r="S194" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO194" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP194" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR194" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS194" t="inlineStr"/>
+      <c r="AT194" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU194" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV194" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW194" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX194" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY194" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ194" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA194" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB194" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC194" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>D007</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>Hepatitis A</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>甲型肝炎</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N195" t="n">
+        <v>7</v>
+      </c>
+      <c r="O195" t="n">
+        <v>7</v>
+      </c>
+      <c r="R195" t="n">
+        <v>0.07771044599357135</v>
+      </c>
+      <c r="S195" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO195" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP195" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR195" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS195" t="inlineStr"/>
+      <c r="AT195" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU195" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV195" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW195" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX195" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY195" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ195" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA195" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB195" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC195" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>D011</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>Hepatitis E</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>戊型肝炎</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N196" t="n">
+        <v>6</v>
+      </c>
+      <c r="O196" t="n">
+        <v>6</v>
+      </c>
+      <c r="R196" t="n">
+        <v>0.06660895370877544</v>
+      </c>
+      <c r="S196" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO196" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP196" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR196" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS196" t="inlineStr"/>
+      <c r="AT196" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU196" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV196" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW196" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX196" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY196" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ196" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA196" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB196" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC196" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>D038</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>Influenza</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>流行性感冒</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N197" t="n">
+        <v>37</v>
+      </c>
+      <c r="O197" t="n">
+        <v>37</v>
+      </c>
+      <c r="R197" t="n">
+        <v>0.4107552145374486</v>
+      </c>
+      <c r="S197" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO197" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP197" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR197" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS197" t="inlineStr"/>
+      <c r="AT197" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU197" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV197" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW197" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX197" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY197" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ197" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA197" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB197" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC197" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>D092</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>Campylobacteriosis</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>弯曲杆菌病</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N198" t="n">
+        <v>1280</v>
+      </c>
+      <c r="O198" t="n">
+        <v>1280</v>
+      </c>
+      <c r="R198" t="n">
+        <v>14.20991012453876</v>
+      </c>
+      <c r="S198" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO198" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP198" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR198" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS198" t="inlineStr"/>
+      <c r="AT198" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU198" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV198" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW198" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX198" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY198" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ198" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA198" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB198" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC198" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>D105</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>Shigellosis</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>志贺菌病</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N199" t="n">
+        <v>22</v>
+      </c>
+      <c r="O199" t="n">
+        <v>22</v>
+      </c>
+      <c r="R199" t="n">
+        <v>0.2442328302655099</v>
+      </c>
+      <c r="S199" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO199" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP199" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR199" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS199" t="inlineStr"/>
+      <c r="AT199" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU199" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV199" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW199" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX199" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY199" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ199" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA199" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB199" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC199" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>D114</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>Salmonellosis</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>沙门氏菌病</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N200" t="n">
+        <v>290</v>
+      </c>
+      <c r="O200" t="n">
+        <v>290</v>
+      </c>
+      <c r="R200" t="n">
+        <v>3.219432762590813</v>
+      </c>
+      <c r="S200" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO200" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP200" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR200" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS200" t="inlineStr"/>
+      <c r="AT200" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU200" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV200" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW200" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX200" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY200" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ200" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA200" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB200" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC200" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N201" t="n">
+        <v>243</v>
+      </c>
+      <c r="O201" t="n">
+        <v>243</v>
+      </c>
+      <c r="R201" t="n">
+        <v>2.697662625205405</v>
+      </c>
+      <c r="S201" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO201" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP201" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR201" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS201" t="inlineStr"/>
+      <c r="AT201" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU201" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV201" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW201" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX201" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY201" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ201" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA201" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB201" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC201" t="inlineStr">
         <is>
           <t>rest_api</t>
         </is>
@@ -29032,7 +30192,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-01</t>
         </is>
       </c>
     </row>
@@ -29115,7 +30275,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="10">
@@ -29125,7 +30285,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11">
@@ -29177,7 +30337,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>48808</v>
+        <v>50786</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-08-21 02:00:34 UTC
</commit_message>
<xml_diff>
--- a/countries/ch/2026-2029.xlsx
+++ b/countries/ch/2026-2029.xlsx
@@ -9587,13 +9587,13 @@
         </is>
       </c>
       <c r="N62" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O62" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R62" t="n">
-        <v>0.05550746142397953</v>
+        <v>0.06660895370877544</v>
       </c>
       <c r="S62" t="inlineStr">
         <is>
@@ -14354,13 +14354,13 @@
         </is>
       </c>
       <c r="N94" t="n">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="O94" t="n">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="R94" t="n">
-        <v>2.908590978616528</v>
+        <v>2.897489486331732</v>
       </c>
       <c r="S94" t="inlineStr">
         <is>
@@ -14934,13 +14934,13 @@
         </is>
       </c>
       <c r="N98" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O98" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R98" t="n">
-        <v>0.06660895370877544</v>
+        <v>0.07771044599357135</v>
       </c>
       <c r="S98" t="inlineStr">
         <is>
@@ -19973,13 +19973,13 @@
         </is>
       </c>
       <c r="N132" t="n">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="O132" t="n">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="R132" t="n">
-        <v>4.362886467924791</v>
+        <v>4.351784975639996</v>
       </c>
       <c r="S132" t="inlineStr">
         <is>
@@ -20553,13 +20553,13 @@
         </is>
       </c>
       <c r="N136" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O136" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R136" t="n">
-        <v>0.1110149228479591</v>
+        <v>0.1332179074175509</v>
       </c>
       <c r="S136" t="inlineStr">
         <is>
@@ -21091,13 +21091,13 @@
         </is>
       </c>
       <c r="N139" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="O139" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="R139" t="n">
-        <v>0.355247753113469</v>
+        <v>0.3774507376830608</v>
       </c>
       <c r="S139" t="inlineStr">
         <is>
@@ -24571,13 +24571,13 @@
         </is>
       </c>
       <c r="N163" t="n">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="O163" t="n">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="R163" t="n">
-        <v>9.702704256911622</v>
+        <v>9.691602764626827</v>
       </c>
       <c r="S163" t="inlineStr">
         <is>
@@ -25151,13 +25151,13 @@
         </is>
       </c>
       <c r="N167" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O167" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="R167" t="n">
-        <v>0.2109283534111222</v>
+        <v>0.2220298456959181</v>
       </c>
       <c r="S167" t="inlineStr">
         <is>
@@ -25296,13 +25296,13 @@
         </is>
       </c>
       <c r="N168" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="O168" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R168" t="n">
-        <v>0.7549014753661216</v>
+        <v>0.7437999830813258</v>
       </c>
       <c r="S168" t="inlineStr">
         <is>
@@ -28196,13 +28196,13 @@
         </is>
       </c>
       <c r="N188" t="n">
-        <v>2143</v>
+        <v>2183</v>
       </c>
       <c r="O188" t="n">
-        <v>2143</v>
+        <v>2183</v>
       </c>
       <c r="R188" t="n">
-        <v>23.79049796631763</v>
+        <v>24.23455765770947</v>
       </c>
       <c r="S188" t="inlineStr">
         <is>
@@ -28776,13 +28776,13 @@
         </is>
       </c>
       <c r="N192" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="O192" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="R192" t="n">
-        <v>0.1665223842719386</v>
+        <v>0.2331313379807141</v>
       </c>
       <c r="S192" t="inlineStr">
         <is>
@@ -28921,13 +28921,13 @@
         </is>
       </c>
       <c r="N193" t="n">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="O193" t="n">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="R193" t="n">
-        <v>1.187859674473162</v>
+        <v>1.365483551029897</v>
       </c>
       <c r="S193" t="inlineStr">
         <is>
@@ -29907,17 +29907,17 @@
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>D114</t>
+          <t>D109</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Salmonellosis</t>
+          <t>Lyme disease</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>沙门氏菌病</t>
+          <t>莱姆病</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -29936,13 +29936,13 @@
         </is>
       </c>
       <c r="N200" t="n">
-        <v>290</v>
+        <v>1746</v>
       </c>
       <c r="O200" t="n">
-        <v>290</v>
+        <v>1746</v>
       </c>
       <c r="R200" t="n">
-        <v>3.219432762590813</v>
+        <v>19.38320552925365</v>
       </c>
       <c r="S200" t="inlineStr">
         <is>
@@ -30052,17 +30052,17 @@
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>D115</t>
+          <t>D114</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Shiga toxin-producing Escherichia coli infection</t>
+          <t>Salmonellosis</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
         <is>
-          <t>产志贺毒素大肠杆菌感染</t>
+          <t>沙门氏菌病</t>
         </is>
       </c>
       <c r="K201" t="inlineStr">
@@ -30081,13 +30081,13 @@
         </is>
       </c>
       <c r="N201" t="n">
-        <v>243</v>
+        <v>290</v>
       </c>
       <c r="O201" t="n">
-        <v>243</v>
+        <v>290</v>
       </c>
       <c r="R201" t="n">
-        <v>2.697662625205405</v>
+        <v>3.219432762590813</v>
       </c>
       <c r="S201" t="inlineStr">
         <is>
@@ -30154,6 +30154,441 @@
         </is>
       </c>
       <c r="BC201" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>D115</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>Shiga toxin-producing Escherichia coli infection</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>产志贺毒素大肠杆菌感染</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N202" t="n">
+        <v>243</v>
+      </c>
+      <c r="O202" t="n">
+        <v>243</v>
+      </c>
+      <c r="R202" t="n">
+        <v>2.697662625205405</v>
+      </c>
+      <c r="S202" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO202" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP202" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR202" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS202" t="inlineStr"/>
+      <c r="AT202" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU202" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV202" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW202" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX202" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY202" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ202" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA202" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB202" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC202" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>D123</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>Tularemia</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>土拉菌病</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N203" t="n">
+        <v>18</v>
+      </c>
+      <c r="O203" t="n">
+        <v>18</v>
+      </c>
+      <c r="R203" t="n">
+        <v>0.1998268611263263</v>
+      </c>
+      <c r="S203" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO203" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP203" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR203" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS203" t="inlineStr"/>
+      <c r="AT203" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU203" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV203" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW203" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX203" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY203" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ203" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA203" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB203" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC203" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>D205</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Tick-borne encephalitis</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>蜱传脑炎</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Viral</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="N204" t="n">
+        <v>101</v>
+      </c>
+      <c r="O204" t="n">
+        <v>101</v>
+      </c>
+      <c r="R204" t="n">
+        <v>1.121250720764387</v>
+      </c>
+      <c r="S204" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO204" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP204" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR204" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS204" t="inlineStr"/>
+      <c r="AT204" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU204" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV204" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="AW204" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="AX204" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="AY204" t="inlineStr">
+        <is>
+          <t>rest_api</t>
+        </is>
+      </c>
+      <c r="AZ204" t="inlineStr">
+        <is>
+          <t>foph_idd</t>
+        </is>
+      </c>
+      <c r="BA204" t="inlineStr">
+        <is>
+          <t>Switzerland FOPH IDD</t>
+        </is>
+      </c>
+      <c r="BB204" t="inlineStr">
+        <is>
+          <t>https://www.idd.bag.admin.ch/en/portal-data</t>
+        </is>
+      </c>
+      <c r="BC204" t="inlineStr">
         <is>
           <t>rest_api</t>
         </is>
@@ -30275,7 +30710,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10">
@@ -30285,7 +30720,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11">
@@ -30337,7 +30772,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>50786</v>
+        <v>52716</v>
       </c>
     </row>
     <row r="16">

</xml_diff>